<commit_message>
Dopunjena projektna dokumentacija za M1
</commit_message>
<xml_diff>
--- a/docs/Majstori_Web_App_dokumentacija.xlsx
+++ b/docs/Majstori_Web_App_dokumentacija.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\users\harun\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E640D68-9338-4530-9E07-E22B4859B490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{865E8F00-371B-4D1F-B66E-CC11F9120E0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-2568" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="97">
   <si>
     <t>Početna dokumentacija projekta</t>
   </si>
@@ -81,7 +81,9 @@
     <t>8. Tehnički koncept projekta</t>
   </si>
   <si>
-    <t>Projekat se razvija kao web aplikacija s frontend dijelom i backend REST API-jem, uz PHP, JavaScript i MySQL. Frontend komunicira s backendom asinhronim AJAX zahtjevima. Backend obrađuje zahtjeve, provjerava pristup i poslovna pravila te komunicira s bazom podataka. Projekat uključuje dokumentaciju API-ja i integraciju vanjskog API-ja, čija će konkretna upotreba biti precizirana tokom razvoja.</t>
+    <t>Projekat se razvija kao web aplikacija s frontend dijelom i backend REST API-jem, uz PHP, JavaScript i MySQL. Frontend komunicira s backendom asinhronim AJAX zahtjevima. Backend obrađuje zahtjeve, provjerava pristup i poslovna pravila te komunicira s bazom podataka. Projekat uključuje dokumentaciju API-ja i integraciju vanjskog API-ja, čija će konkretna upotreba biti precizirana tokom razvoja.
+Trenutni frontend: HTML, CSS, JavaScript i jQuery. Planirane backend tehnologije: PHP, FlightPHP, MySQL, PDO, REST API i JWT; nisu sve još implementirane.
+Planirana integracija: Nominatim za pronalaženje geografskih koordinata i OpenStreetMap za prikaz lokacije na mapi.</t>
   </si>
   <si>
     <t>9. Status dokumenta</t>
@@ -90,6 +92,12 @@
     <t>Ovaj opis predstavlja početnu verziju nastalu na osnovu dosadašnje analize zahtjeva. Nije konačna specifikacija: sadržaj se može mijenjati, dopunjavati i precizirati tokom razvoja, testiranja i dogovaranja detalja projekta.</t>
   </si>
   <si>
+    <t>Dodatno pojašnjenje – administratorski račun</t>
+  </si>
+  <si>
+    <t>Administrator nema vlastiti profil majstora. Može pregledati određene podatke profila majstora samo za čitanje, bez uređivanja profila ili upravljanja odabranim majstorlucima kroz taj prikaz.</t>
+  </si>
+  <si>
     <t>MAJSTORI WEB APP — REGISTAR POSLOVNIH PRAVILA</t>
   </si>
   <si>
@@ -159,78 +167,78 @@
     <t>Majstor može promijeniti svoju lozinku. Sistem pohranjuje hash lozinke, a ne lozinku u čitljivom obliku.</t>
   </si>
   <si>
+    <t>Profil majstora</t>
+  </si>
+  <si>
+    <t>P003</t>
+  </si>
+  <si>
+    <t>Majstor uređuje vlastiti profil</t>
+  </si>
+  <si>
+    <t>Nakon uspješne prijave.</t>
+  </si>
+  <si>
+    <t>Majstor može urediti podatke svog profila, uključujući ime, prezime, kontaktni telefon, opis usluga i grad u kojem posluje.</t>
+  </si>
+  <si>
+    <t>P004</t>
+  </si>
+  <si>
+    <t>Majstor bira kategorije usluga</t>
+  </si>
+  <si>
+    <t>Prilikom uređivanja vlastitog profila.</t>
+  </si>
+  <si>
+    <t>Majstor može odabrati kategorije usluga iz hijerarhijskog stabla majstorluka. Odabir se čuva kao direktna veza majstora s odabranom kategorijom; odabir roditeljske kategorije ne znači automatski odabir svih njenih potkategorija.</t>
+  </si>
+  <si>
+    <t>Gradovi i profil majstora</t>
+  </si>
+  <si>
+    <t>P005</t>
+  </si>
+  <si>
+    <t>Majstor bira grad iz administratorske liste</t>
+  </si>
+  <si>
+    <t>Majstor bira grad iz liste gradova koje je administrator prethodno unio. Ne unosi proizvoljan naziv grada niti koordinate. Sistem koristi sačuvane koordinate grada za približnu lokacijsku pretragu. Aplikacija je namijenjena području Bosne i Hercegovine.</t>
+  </si>
+  <si>
+    <t>Administracija kategorija</t>
+  </si>
+  <si>
+    <t>P007</t>
+  </si>
+  <si>
+    <t>Admin upravlja stablom majstorluka</t>
+  </si>
+  <si>
+    <t>Kada je prijavljen kao administrator.</t>
+  </si>
+  <si>
+    <t>Administrator može dodavati kategorije, mijenjati njihove nazive, premještati ih pod drugu kategoriju i brisati kategorije u skladu s validacijama navedenim u ovom registru.</t>
+  </si>
+  <si>
+    <t>P008</t>
+  </si>
+  <si>
+    <t>Premještanje ne mijenja direktne odabire majstora</t>
+  </si>
+  <si>
+    <t>Kada administrator premjesti kategoriju u drugi dio stabla.</t>
+  </si>
+  <si>
+    <t>Premještanje mijenja samo roditeljsku vezu kategorije. Zapisi u majstor_kategorije ostaju isti. Rezultati pretrage po roditeljskim kategorijama ipak se mogu promijeniti jer se mijenja hijerarhija.</t>
+  </si>
+  <si>
+    <t>V001</t>
+  </si>
+  <si>
     <t>Validacija</t>
   </si>
   <si>
-    <t>Profil majstora</t>
-  </si>
-  <si>
-    <t>P003</t>
-  </si>
-  <si>
-    <t>Majstor uređuje vlastiti profil</t>
-  </si>
-  <si>
-    <t>Nakon uspješne prijave.</t>
-  </si>
-  <si>
-    <t>Majstor može urediti podatke svog profila, uključujući ime, prezime, kontaktni telefon, opis usluga i grad u kojem posluje.</t>
-  </si>
-  <si>
-    <t>P004</t>
-  </si>
-  <si>
-    <t>Majstor bira kategorije usluga</t>
-  </si>
-  <si>
-    <t>Prilikom uređivanja vlastitog profila.</t>
-  </si>
-  <si>
-    <t>Majstor može odabrati kategorije usluga iz hijerarhijskog stabla majstorluka. Odabir se čuva kao direktna veza majstora s odabranom kategorijom; odabir roditeljske kategorije ne znači automatski odabir svih njenih potkategorija.</t>
-  </si>
-  <si>
-    <t>Gradovi i profil majstora</t>
-  </si>
-  <si>
-    <t>P005</t>
-  </si>
-  <si>
-    <t>Majstor bira grad iz administratorske liste</t>
-  </si>
-  <si>
-    <t>Majstor bira grad iz liste gradova koje je administrator prethodno unio. Ne unosi proizvoljan naziv grada niti koordinate. Sistem koristi sačuvane koordinate grada za približnu lokacijsku pretragu. Aplikacija je namijenjena području Bosne i Hercegovine.</t>
-  </si>
-  <si>
-    <t>Administracija kategorija</t>
-  </si>
-  <si>
-    <t>P007</t>
-  </si>
-  <si>
-    <t>Admin upravlja stablom majstorluka</t>
-  </si>
-  <si>
-    <t>Kada je prijavljen kao administrator.</t>
-  </si>
-  <si>
-    <t>Administrator može dodavati kategorije, mijenjati njihove nazive, premještati ih pod drugu kategoriju i brisati kategorije u skladu s validacijama navedenim u ovom registru.</t>
-  </si>
-  <si>
-    <t>P008</t>
-  </si>
-  <si>
-    <t>Premještanje ne mijenja direktne odabire majstora</t>
-  </si>
-  <si>
-    <t>Kada administrator premjesti kategoriju u drugi dio stabla.</t>
-  </si>
-  <si>
-    <t>Premještanje mijenja samo roditeljsku vezu kategorije. Zapisi u majstor_kategorije ostaju isti. Rezultati pretrage po roditeljskim kategorijama ipak se mogu promijeniti jer se mijenja hijerarhija.</t>
-  </si>
-  <si>
-    <t>V001</t>
-  </si>
-  <si>
     <t>Brisati se mogu samo kategorije-listovi</t>
   </si>
   <si>
@@ -304,18 +312,6 @@
   </si>
   <si>
     <t>Aplikacija prikazuje naziv grada i lokaciju koju je pronašao unaprijed pripremljeni izvor podataka/geocoding servis. Administrator potvrđuje da je riječ o željenom gradu u Bosni i Hercegovini. Grad se ne sprema ako odgovarajući rezultat nije pronađen ili ako administrator ne potvrdi lokaciju.</t>
-  </si>
-  <si>
-    <t>V005</t>
-  </si>
-  <si>
-    <t>Ne uklanjati grad koji koriste profili majstora</t>
-  </si>
-  <si>
-    <t>Prije brisanja grada.</t>
-  </si>
-  <si>
-    <t>Backend provjerava da li je grad povezan s nekim profilom majstora. Ako jeste, brisanje se odbija dok se profili ne prebace na drugi grad. Time se izbjegava gubitak veze između profila majstora i grada.</t>
   </si>
   <si>
     <r>
@@ -325,24 +321,13 @@
     <r>
       <rPr>
         <b/>
-        <sz val="18"/>
-        <color theme="4" tint="-0.249977111117893"/>
+        <sz val="16"/>
+        <color rgb="FF0070C0"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>„Opis_aplikacije“</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="18"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  
-</t>
+      <t xml:space="preserve">„Opis_aplikacije“ </t>
     </r>
     <r>
       <rPr>
@@ -351,24 +336,15 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>u kojem su predstavljeni namjena, korisnici i osnovne funkcionalnosti aplikacije
+      <t xml:space="preserve"> 
+u kojem su predstavljeni namjena, korisnici i osnovne funkcionalnosti aplikacije
 i
-Sheet</t>
+Sheet </t>
     </r>
     <r>
       <rPr>
         <b/>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="18"/>
+        <sz val="16"/>
         <color rgb="FF00B050"/>
         <rFont val="Calibri"/>
         <family val="2"/>
@@ -378,47 +354,25 @@
     </r>
     <r>
       <rPr>
-        <b/>
-        <sz val="18"/>
+        <sz val="12"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
+u kojem su detaljnije razrađena pravila, validacije i akcije sistema
 </t>
     </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">u kojem su detaljnije razrađena pravila, validacije i akcije sistema
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">MAJSTORI WEB APP  </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="16"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>- Harun Tabak, 2026.</t>
-    </r>
+  </si>
+  <si>
+    <t>MAJSTORI WEB APP  - Harun Tabak, IBU, 2026.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -480,13 +434,6 @@
     </font>
     <font>
       <b/>
-      <sz val="18"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="10"/>
       <color rgb="FF1F1F1F"/>
       <name val="Calibri"/>
@@ -501,38 +448,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="14"/>
       <color rgb="FF666666"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="4" tint="-0.249977111117893"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -542,6 +459,22 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -607,7 +540,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -633,13 +566,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -669,30 +602,34 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1009,36 +946,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
-        <v>98</v>
-      </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
+      <c r="A1" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
     </row>
     <row r="2" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="24"/>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
+      <c r="A2" s="21"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
     </row>
     <row r="4" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
     </row>
     <row r="6" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="20" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B6" s="21"/>
       <c r="C6" s="21"/>
@@ -1104,285 +1041,284 @@
   <sheetPr>
     <tabColor theme="4" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
     </row>
     <row r="3" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
     </row>
     <row r="4" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
     </row>
     <row r="5" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="24"/>
-      <c r="B5" s="24"/>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
+      <c r="A5" s="27"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
     </row>
     <row r="7" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="26" t="s">
+      <c r="A7" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
     </row>
     <row r="8" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="24"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
     </row>
     <row r="9" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="24"/>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
+      <c r="A9" s="27"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
     </row>
     <row r="11" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="26" t="s">
+      <c r="A11" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="24"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
     </row>
     <row r="12" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="27" t="s">
+      <c r="A12" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="24"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
     </row>
     <row r="13" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="24"/>
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
+      <c r="A13" s="27"/>
+      <c r="B13" s="27"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
     </row>
     <row r="15" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="26" t="s">
+      <c r="A15" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
     </row>
     <row r="16" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="21"/>
     </row>
     <row r="17" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="24"/>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
+      <c r="A17" s="27"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
     </row>
     <row r="19" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="26" t="s">
+      <c r="A19" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
     </row>
     <row r="20" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="27" t="s">
+      <c r="A20" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
     </row>
     <row r="21" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="24"/>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
+      <c r="A21" s="27"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
     </row>
     <row r="23" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="26" t="s">
+      <c r="A23" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
     </row>
     <row r="24" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="27" t="s">
+      <c r="A24" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
     </row>
     <row r="25" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="24"/>
-      <c r="B25" s="24"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
+      <c r="A25" s="27"/>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
     </row>
     <row r="27" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="26" t="s">
+      <c r="A27" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="24"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
     </row>
     <row r="28" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="27" t="s">
+      <c r="A28" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B28" s="24"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
     </row>
     <row r="29" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="24"/>
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
+      <c r="A29" s="27"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="27"/>
     </row>
     <row r="31" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="26" t="s">
+      <c r="A31" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="B31" s="24"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="24"/>
-      <c r="F31" s="24"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
     </row>
     <row r="32" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="27" t="s">
+      <c r="A32" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="B32" s="24"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="24"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="21"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
     </row>
     <row r="33" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="24"/>
-      <c r="B33" s="24"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
+      <c r="A33" s="27"/>
+      <c r="B33" s="27"/>
+      <c r="C33" s="27"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="27"/>
     </row>
     <row r="35" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="26" t="s">
+      <c r="A35" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="B35" s="24"/>
-      <c r="C35" s="24"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="24"/>
-      <c r="F35" s="24"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="21"/>
+      <c r="D35" s="21"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="21"/>
     </row>
     <row r="36" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="27" t="s">
+      <c r="A36" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="B36" s="24"/>
-      <c r="C36" s="24"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="24"/>
-      <c r="F36" s="24"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
     </row>
     <row r="37" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="24"/>
-      <c r="B37" s="24"/>
-      <c r="C37" s="24"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="24"/>
-      <c r="F37" s="24"/>
+      <c r="A37" s="27"/>
+      <c r="B37" s="27"/>
+      <c r="C37" s="27"/>
+      <c r="D37" s="27"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="27"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>21</v>
+      </c>
+      <c r="B38" t="s">
+        <v>22</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A8:F9"/>
-    <mergeCell ref="A4:F5"/>
-    <mergeCell ref="A20:F21"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A12:F13"/>
-    <mergeCell ref="A15:F15"/>
-    <mergeCell ref="A11:F11"/>
     <mergeCell ref="A35:F35"/>
     <mergeCell ref="A36:F37"/>
     <mergeCell ref="A16:F17"/>
@@ -1393,6 +1329,15 @@
     <mergeCell ref="A28:F29"/>
     <mergeCell ref="A23:F23"/>
     <mergeCell ref="A24:F25"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A8:F9"/>
+    <mergeCell ref="A4:F5"/>
+    <mergeCell ref="A20:F21"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A12:F13"/>
+    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A11:F11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1416,358 +1361,346 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
-        <v>21</v>
-      </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
+      <c r="A1" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="21"/>
     </row>
     <row r="2" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
+      <c r="A2" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="21"/>
     </row>
     <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
+        <v>25</v>
+      </c>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="21"/>
     </row>
     <row r="4" spans="1:7" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:7" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="D20" s="18" t="s">
-        <v>94</v>
-      </c>
-      <c r="E20" s="18" t="s">
-        <v>95</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>96</v>
-      </c>
+      <c r="A20" s="2"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
     </row>
   </sheetData>
   <autoFilter ref="A5:F20" xr:uid="{00000000-0009-0000-0000-000002000000}"/>

</xml_diff>